<commit_message>
Added warehouse dashboard and order status management
</commit_message>
<xml_diff>
--- a/output/order_data.xlsx
+++ b/output/order_data.xlsx
@@ -16,11 +16,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
-    <numFmt numFmtId="166" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="167" formatCode="YYYY-MM-DD"/>
   </numFmts>
   <fonts count="2">
     <font>
@@ -60,13 +58,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -432,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:I4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -513,16 +510,16 @@
       </c>
       <c r="G2" t="inlineStr"/>
       <c r="H2" s="2" t="n">
-        <v>46207</v>
+        <v>46209</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>46207</v>
+        <v>46209</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>ORD0002</t>
+          <t>ORD0001</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -550,16 +547,16 @@
       </c>
       <c r="G3" t="inlineStr"/>
       <c r="H3" s="2" t="n">
-        <v>46207</v>
+        <v>46209</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>46207</v>
+        <v>46209</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>ORD0003</t>
+          <t>ORD0002</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -569,7 +566,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>LAPTOP</t>
+          <t>laptop</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -577,7 +574,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>allocated</t>
+          <t>Picking</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -586,48 +583,11 @@
         </is>
       </c>
       <c r="G4" t="inlineStr"/>
-      <c r="H4" s="3" t="n">
-        <v>46207</v>
-      </c>
-      <c r="I4" s="3" t="n">
-        <v>46207</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>ORD0003</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>WH005</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>mouse</t>
-        </is>
-      </c>
-      <c r="D5" t="n">
-        <v>1</v>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>allocated</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>Bengaluru</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" s="3" t="n">
-        <v>46207</v>
-      </c>
-      <c r="I5" s="3" t="n">
-        <v>46207</v>
+      <c r="H4" s="2" t="n">
+        <v>46209</v>
+      </c>
+      <c r="I4" s="2" t="n">
+        <v>46209</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
now advancing to sql
</commit_message>
<xml_diff>
--- a/output/order_data.xlsx
+++ b/output/order_data.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:I6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -588,6 +588,80 @@
       </c>
       <c r="I4" s="2" t="n">
         <v>46209</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>ORD0003</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>WH005</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>sanitizer</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Picking</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Bengaluru</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" s="2" t="n">
+        <v>46210</v>
+      </c>
+      <c r="I5" s="2" t="n">
+        <v>46210</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>ORD0003</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>WH005</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>backpack</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Picking</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Bengaluru</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" s="2" t="n">
+        <v>46210</v>
+      </c>
+      <c r="I6" s="2" t="n">
+        <v>46210</v>
       </c>
     </row>
   </sheetData>

</xml_diff>